<commit_message>
Say department, office or RM in the descriptions, not unit
Unit is the third level of the ADB hierarchy Fred settled in the
technical sync, and the level the report does not use. Fifty-five
descriptions used it loosely to mean the thing that owns the row or
the thing the picker selects, which reads as the wrong hierarchy level.

Bank-wide spells the owner out on all six affected rows. Department
Insights defines the selected department once, on the picker item,
and uses it in the forty-nine below.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VdkbQVuogqce5Eq5woYD3Q
</commit_message>
<xml_diff>
--- a/EDRMS_Utilization_Dashboard_Checker_with_Description.xlsx
+++ b/EDRMS_Utilization_Dashboard_Checker_with_Description.xlsx
@@ -11149,7 +11149,7 @@
       </c>
       <c r="D18" s="67" t="inlineStr">
         <is>
-          <t>The first column of the site table. One row per owning unit, so units can be compared side by side.</t>
+          <t>The first column of the site table. One row per owning department, office or RM, so they can be compared side by side.</t>
         </is>
       </c>
       <c r="E18" s="40" t="inlineStr">
@@ -11180,7 +11180,7 @@
       </c>
       <c r="D19" s="82" t="inlineStr">
         <is>
-          <t>For the one unit on that row: how many EDRMS sites it owns.</t>
+          <t>For the one department, office or RM on that row: how many EDRMS sites it owns.</t>
         </is>
       </c>
       <c r="E19" s="43" t="inlineStr">
@@ -11211,7 +11211,7 @@
       </c>
       <c r="D20" s="67" t="inlineStr">
         <is>
-          <t>For the one unit on that row: every document held across that unit's EDRMS sites.</t>
+          <t>For the one department, office or RM on that row: every document held across that row's EDRMS sites.</t>
         </is>
       </c>
       <c r="E20" s="40" t="inlineStr">
@@ -11242,7 +11242,7 @@
       </c>
       <c r="D21" s="82" t="inlineStr">
         <is>
-          <t>For the one unit on that row: how many of its documents have been declared as records.</t>
+          <t>For the one department, office or RM on that row: how many of its documents have been declared as records.</t>
         </is>
       </c>
       <c r="E21" s="43" t="inlineStr">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="D22" s="67" t="inlineStr">
         <is>
-          <t>For the one unit on that row: how many of its declared records also exist on paper.</t>
+          <t>For the one department, office or RM on that row: how many of its declared records also exist on paper.</t>
         </is>
       </c>
       <c r="E22" s="40" t="inlineStr">
@@ -12755,7 +12755,7 @@
       </c>
       <c r="D74" s="67" t="inlineStr">
         <is>
-          <t>A comparison showing, for each unit, how many documents it holds against how many it has declared.</t>
+          <t>A comparison showing, for each department, office or RM, how many documents it holds against how many it has declared.</t>
         </is>
       </c>
       <c r="E74" s="40" t="inlineStr">
@@ -21256,7 +21256,7 @@
       </c>
       <c r="D7" s="40" t="inlineStr">
         <is>
-          <t>Not a figure. The control that chooses which department, office or RM the whole screen is about.</t>
+          <t>Not a figure. The control that chooses which department, office or RM the whole screen is about. Every figure below is for that one choice only, called 'the selected department' throughout this column.</t>
         </is>
       </c>
       <c r="E7" s="40" t="inlineStr">
@@ -21287,7 +21287,7 @@
       </c>
       <c r="D8" s="43" t="inlineStr">
         <is>
-          <t>How many EDRMS sites the selected unit owns.</t>
+          <t>How many EDRMS sites the selected department owns.</t>
         </is>
       </c>
       <c r="E8" s="43" t="inlineStr">
@@ -21318,7 +21318,7 @@
       </c>
       <c r="D9" s="40" t="inlineStr">
         <is>
-          <t>How many people count as EDRMS users for the selected unit.</t>
+          <t>How many people count as EDRMS users for the selected department.</t>
         </is>
       </c>
       <c r="E9" s="40" t="inlineStr">
@@ -21349,7 +21349,7 @@
       </c>
       <c r="D10" s="43" t="inlineStr">
         <is>
-          <t>How many people visited the selected unit's EDRMS sites.</t>
+          <t>How many people visited the selected department's EDRMS sites.</t>
         </is>
       </c>
       <c r="E10" s="43" t="inlineStr">
@@ -21380,7 +21380,7 @@
       </c>
       <c r="D11" s="40" t="inlineStr">
         <is>
-          <t>Every document held across the selected unit's EDRMS sites, declared or not.</t>
+          <t>Every document held across the selected department's EDRMS sites, declared or not.</t>
         </is>
       </c>
       <c r="E11" s="40" t="inlineStr">
@@ -21411,7 +21411,7 @@
       </c>
       <c r="D12" s="43" t="inlineStr">
         <is>
-          <t>How many of the selected unit's documents have been declared as records.</t>
+          <t>How many of the selected department's documents have been declared as records.</t>
         </is>
       </c>
       <c r="E12" s="43" t="inlineStr">
@@ -21442,7 +21442,7 @@
       </c>
       <c r="D13" s="40" t="inlineStr">
         <is>
-          <t>How many of the selected unit's declared records also exist on paper.</t>
+          <t>How many of the selected department's declared records also exist on paper.</t>
         </is>
       </c>
       <c r="E13" s="40" t="inlineStr">
@@ -21473,7 +21473,7 @@
       </c>
       <c r="D14" s="43" t="inlineStr">
         <is>
-          <t>How many of the selected unit's records reach their disposal due date.</t>
+          <t>How many of the selected department's records reach their disposal due date.</t>
         </is>
       </c>
       <c r="E14" s="43" t="inlineStr">
@@ -21531,7 +21531,7 @@
       </c>
       <c r="D16" s="43" t="inlineStr">
         <is>
-          <t>The naming rules the selected unit's sites, libraries and folders are meant to follow.</t>
+          <t>The naming rules the selected department's sites, libraries and folders are meant to follow.</t>
         </is>
       </c>
       <c r="E16" s="43" t="inlineStr">
@@ -21562,7 +21562,7 @@
       </c>
       <c r="D17" s="40" t="inlineStr">
         <is>
-          <t>The date the selected unit started using EDRMS.</t>
+          <t>The date the selected department started using EDRMS.</t>
         </is>
       </c>
       <c r="E17" s="40" t="inlineStr">
@@ -21606,7 +21606,7 @@
       </c>
       <c r="D19" s="43" t="inlineStr">
         <is>
-          <t>How many of the selected unit's people have used EDRMS recently.</t>
+          <t>How many of the selected department's people have used EDRMS recently.</t>
         </is>
       </c>
       <c r="E19" s="43" t="inlineStr">
@@ -21637,7 +21637,7 @@
       </c>
       <c r="D20" s="40" t="inlineStr">
         <is>
-          <t>How many of the selected unit's people opened EDRMS in the last 180 days.</t>
+          <t>How many of the selected department's people opened EDRMS in the last 180 days.</t>
         </is>
       </c>
       <c r="E20" s="40" t="inlineStr">
@@ -21699,7 +21699,7 @@
       </c>
       <c r="D22" s="40" t="inlineStr">
         <is>
-          <t>How many of the selected unit's people have access to an EDRMS site but have never once opened it.</t>
+          <t>How many of the selected department's people have access to an EDRMS site but have never once opened it.</t>
         </is>
       </c>
       <c r="E22" s="40" t="inlineStr">
@@ -21730,7 +21730,7 @@
       </c>
       <c r="D23" s="43" t="inlineStr">
         <is>
-          <t>Of the selected unit's EDRMS users, how many are ADB staff.</t>
+          <t>Of the selected department's EDRMS users, how many are ADB staff.</t>
         </is>
       </c>
       <c r="E23" s="43" t="inlineStr">
@@ -21761,7 +21761,7 @@
       </c>
       <c r="D24" s="40" t="inlineStr">
         <is>
-          <t>Of the selected unit's EDRMS users, how many are contractors.</t>
+          <t>Of the selected department's EDRMS users, how many are contractors.</t>
         </is>
       </c>
       <c r="E24" s="40" t="inlineStr">
@@ -21792,7 +21792,7 @@
       </c>
       <c r="D25" s="43" t="inlineStr">
         <is>
-          <t>Of the selected unit's EDRMS users, how many are consultants.</t>
+          <t>Of the selected department's EDRMS users, how many are consultants.</t>
         </is>
       </c>
       <c r="E25" s="43" t="inlineStr">
@@ -21823,7 +21823,7 @@
       </c>
       <c r="D26" s="40" t="inlineStr">
         <is>
-          <t>What share of the selected unit's EDRMS users have completed EDRMS training.</t>
+          <t>What share of the selected department's EDRMS users have completed EDRMS training.</t>
         </is>
       </c>
       <c r="E26" s="40" t="inlineStr">
@@ -21867,7 +21867,7 @@
       </c>
       <c r="D28" s="43" t="inlineStr">
         <is>
-          <t>How many EDRMS sites the selected unit owns, shown above its site table.</t>
+          <t>How many EDRMS sites the selected department owns, shown above its site table.</t>
         </is>
       </c>
       <c r="E28" s="43" t="inlineStr">
@@ -21898,7 +21898,7 @@
       </c>
       <c r="D29" s="40" t="inlineStr">
         <is>
-          <t>Every document across the selected unit's sites, shown above its site table.</t>
+          <t>Every document across the selected department's sites, shown above its site table.</t>
         </is>
       </c>
       <c r="E29" s="40" t="inlineStr">
@@ -21929,7 +21929,7 @@
       </c>
       <c r="D30" s="43" t="inlineStr">
         <is>
-          <t>Records declared across the selected unit's sites.</t>
+          <t>Records declared across the selected department's sites.</t>
         </is>
       </c>
       <c r="E30" s="43" t="inlineStr">
@@ -21960,7 +21960,7 @@
       </c>
       <c r="D31" s="40" t="inlineStr">
         <is>
-          <t>Paper counterparts across the selected unit's sites.</t>
+          <t>Paper counterparts across the selected department's sites.</t>
         </is>
       </c>
       <c r="E31" s="40" t="inlineStr">
@@ -21991,7 +21991,7 @@
       </c>
       <c r="D32" s="43" t="inlineStr">
         <is>
-          <t>Records in the selected unit falling due for disposal within the next 12 months.</t>
+          <t>Records in the selected department falling due for disposal within the next 12 months.</t>
         </is>
       </c>
       <c r="E32" s="43" t="inlineStr">
@@ -22022,7 +22022,7 @@
       </c>
       <c r="D33" s="40" t="inlineStr">
         <is>
-          <t>One row per site. The name of each EDRMS site the selected unit owns.</t>
+          <t>One row per site. The name of each EDRMS site the selected department owns.</t>
         </is>
       </c>
       <c r="E33" s="40" t="inlineStr">
@@ -22221,7 +22221,7 @@
       </c>
       <c r="D40" s="40" t="inlineStr">
         <is>
-          <t>How many people visited the selected unit's EDRMS sites.</t>
+          <t>How many people visited the selected department's EDRMS sites.</t>
         </is>
       </c>
       <c r="E40" s="40" t="inlineStr">
@@ -22252,7 +22252,7 @@
       </c>
       <c r="D41" s="43" t="inlineStr">
         <is>
-          <t>A table showing visit activity for each of the selected unit's sites.</t>
+          <t>A table showing visit activity for each of the selected department's sites.</t>
         </is>
       </c>
       <c r="E41" s="43" t="inlineStr">
@@ -22283,7 +22283,7 @@
       </c>
       <c r="D42" s="40" t="inlineStr">
         <is>
-          <t>How many pages were viewed in total across the selected unit's sites.</t>
+          <t>How many pages were viewed in total across the selected department's sites.</t>
         </is>
       </c>
       <c r="E42" s="40" t="inlineStr">
@@ -22523,7 +22523,7 @@
       </c>
       <c r="D50" s="40" t="inlineStr">
         <is>
-          <t>Of the people who visited the selected unit's sites, how many came from outside ADB.</t>
+          <t>Of the people who visited the selected department's sites, how many came from outside ADB.</t>
         </is>
       </c>
       <c r="E50" s="40" t="inlineStr">
@@ -22554,7 +22554,7 @@
       </c>
       <c r="D51" s="43" t="inlineStr">
         <is>
-          <t>Of the people who visited the selected unit's sites, how many came from inside ADB.</t>
+          <t>Of the people who visited the selected department's sites, how many came from inside ADB.</t>
         </is>
       </c>
       <c r="E51" s="43" t="inlineStr">
@@ -22585,7 +22585,7 @@
       </c>
       <c r="D52" s="40" t="inlineStr">
         <is>
-          <t>How many requests to join the selected unit's sites were approved.</t>
+          <t>How many requests to join the selected department's sites were approved.</t>
         </is>
       </c>
       <c r="E52" s="40" t="inlineStr">
@@ -22616,7 +22616,7 @@
       </c>
       <c r="D53" s="43" t="inlineStr">
         <is>
-          <t>How many requests to join the selected unit's sites were refused.</t>
+          <t>How many requests to join the selected department's sites were refused.</t>
         </is>
       </c>
       <c r="E53" s="43" t="inlineStr">
@@ -22660,7 +22660,7 @@
       </c>
       <c r="D55" s="40" t="inlineStr">
         <is>
-          <t>How many documents have been put into the selected unit's sites.</t>
+          <t>How many documents have been put into the selected department's sites.</t>
         </is>
       </c>
       <c r="E55" s="40" t="inlineStr">
@@ -22691,7 +22691,7 @@
       </c>
       <c r="D56" s="43" t="inlineStr">
         <is>
-          <t>How many of the selected unit's EDRMS sites are currently active.</t>
+          <t>How many of the selected department's EDRMS sites are currently active.</t>
         </is>
       </c>
       <c r="E56" s="43" t="inlineStr">
@@ -22722,7 +22722,7 @@
       </c>
       <c r="D57" s="40" t="inlineStr">
         <is>
-          <t>How much storage space the selected unit's documents occupy.</t>
+          <t>How much storage space the selected department's documents occupy.</t>
         </is>
       </c>
       <c r="E57" s="40" t="inlineStr">
@@ -22846,7 +22846,7 @@
       </c>
       <c r="D61" s="40" t="inlineStr">
         <is>
-          <t>How many distinct people created documents in the selected unit's sites.</t>
+          <t>How many distinct people created documents in the selected department's sites.</t>
         </is>
       </c>
       <c r="E61" s="40" t="inlineStr">
@@ -22890,7 +22890,7 @@
       </c>
       <c r="D63" s="43" t="inlineStr">
         <is>
-          <t>Records declared across the selected unit's sites.</t>
+          <t>Records declared across the selected department's sites.</t>
         </is>
       </c>
       <c r="E63" s="43" t="inlineStr">
@@ -22921,7 +22921,7 @@
       </c>
       <c r="D64" s="40" t="inlineStr">
         <is>
-          <t>How many distinct people in the selected unit declared at least one record.</t>
+          <t>How many distinct people in the selected department declared at least one record.</t>
         </is>
       </c>
       <c r="E64" s="40" t="inlineStr">
@@ -22952,7 +22952,7 @@
       </c>
       <c r="D65" s="43" t="inlineStr">
         <is>
-          <t>Which of the selected unit's sites have had no record declared in the last 180 days.</t>
+          <t>Which of the selected department's sites have had no record declared in the last 180 days.</t>
         </is>
       </c>
       <c r="E65" s="43" t="inlineStr">
@@ -23045,7 +23045,7 @@
       </c>
       <c r="D68" s="40" t="inlineStr">
         <is>
-          <t>How much storage space the selected unit's declared records occupy.</t>
+          <t>How much storage space the selected department's declared records occupy.</t>
         </is>
       </c>
       <c r="E68" s="40" t="inlineStr">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="D72" s="43" t="inlineStr">
         <is>
-          <t>How many of the selected unit's declared records also exist on paper.</t>
+          <t>How many of the selected department's declared records also exist on paper.</t>
         </is>
       </c>
       <c r="E72" s="43" t="inlineStr">
@@ -23182,7 +23182,7 @@
       </c>
       <c r="D73" s="40" t="inlineStr">
         <is>
-          <t>The selected unit's total declared records, shown alongside for comparison.</t>
+          <t>The selected department's total declared records, shown alongside for comparison.</t>
         </is>
       </c>
       <c r="E73" s="40" t="inlineStr">
@@ -23337,7 +23337,7 @@
       </c>
       <c r="D78" s="43" t="inlineStr">
         <is>
-          <t>Of the selected unit's paper counterparts, how many have been handed over to RAC.</t>
+          <t>Of the selected department's paper counterparts, how many have been handed over to RAC.</t>
         </is>
       </c>
       <c r="E78" s="43" t="inlineStr">
@@ -23381,7 +23381,7 @@
       </c>
       <c r="D80" s="40" t="inlineStr">
         <is>
-          <t>Records in the selected unit falling due for disposal within the next 3 months.</t>
+          <t>Records in the selected department falling due for disposal within the next 3 months.</t>
         </is>
       </c>
       <c r="E80" s="40" t="inlineStr">
@@ -23412,7 +23412,7 @@
       </c>
       <c r="D81" s="43" t="inlineStr">
         <is>
-          <t>Records in the selected unit falling due for disposal within the next 6 months.</t>
+          <t>Records in the selected department falling due for disposal within the next 6 months.</t>
         </is>
       </c>
       <c r="E81" s="43" t="inlineStr">
@@ -23443,7 +23443,7 @@
       </c>
       <c r="D82" s="40" t="inlineStr">
         <is>
-          <t>Records in the selected unit falling due for disposal within the next 12 months.</t>
+          <t>Records in the selected department falling due for disposal within the next 12 months.</t>
         </is>
       </c>
       <c r="E82" s="40" t="inlineStr">
@@ -23567,7 +23567,7 @@
       </c>
       <c r="D86" s="40" t="inlineStr">
         <is>
-          <t>Who approved each disposal in the selected unit.</t>
+          <t>Who approved each disposal in the selected department.</t>
         </is>
       </c>
       <c r="E86" s="40" t="inlineStr">
@@ -23598,7 +23598,7 @@
       </c>
       <c r="D87" s="43" t="inlineStr">
         <is>
-          <t>How many disposal requests in the selected unit were approved.</t>
+          <t>How many disposal requests in the selected department were approved.</t>
         </is>
       </c>
       <c r="E87" s="43" t="inlineStr">
@@ -23629,7 +23629,7 @@
       </c>
       <c r="D88" s="40" t="inlineStr">
         <is>
-          <t>How many disposal requests in the selected unit were declined.</t>
+          <t>How many disposal requests in the selected department were declined.</t>
         </is>
       </c>
       <c r="E88" s="40" t="inlineStr">
@@ -23691,7 +23691,7 @@
       </c>
       <c r="D90" s="40" t="inlineStr">
         <is>
-          <t>How many of the selected unit's records were actually disposed, by month and year.</t>
+          <t>How many of the selected department's records were actually disposed, by month and year.</t>
         </is>
       </c>
       <c r="E90" s="40" t="inlineStr">
@@ -23766,7 +23766,7 @@
       </c>
       <c r="D93" s="40" t="inlineStr">
         <is>
-          <t>One row per library. The name of each library inside the selected unit's sites.</t>
+          <t>One row per library. The name of each library inside the selected department's sites.</t>
         </is>
       </c>
       <c r="E93" s="40" t="inlineStr">
@@ -23984,7 +23984,7 @@
       </c>
       <c r="D101" s="43" t="inlineStr">
         <is>
-          <t>The key dates in the EDRMS rollout programme for the selected unit.</t>
+          <t>The key dates in the EDRMS rollout programme for the selected department.</t>
         </is>
       </c>
       <c r="E101" s="43" t="n"/>

</xml_diff>